<commit_message>
Tambah Sheet fokus Baseline vs ABSA Concat+Confidence di laporan Excel
Sheet baru '2_Baseline_vs_Concat_Confidence' (tier Wajib) mengisolasi
perbandingan klaim inti penelitian -- RMSE, MAE, signifikansi, DAN
stabilitas dari baseline vs varian terbaik dalam satu tabel + chart,
tanpa perlu loncat antar Sheet 3 (Hasil Utama)/5 (Signifikansi)/6
(Stabilitas) yang masing-masing mencampur 7 model. Sheet lain di-renumber
(3-8, tier Wajib jadi Sheet 1-4, Lampiran jadi Sheet 5-8); TOC & hyperlink
Sheet 0 diupdate mengikuti. Sheet 3 (bekas Sheet 2) diverifikasi ulang
21/21 baris tetap cocok dgn manuscript_table_*.csv setelah renumbering.

Tambah .gitignore rule utk file lock sementara MS Office (~$*.xlsx dst) --
sempat muncul stray file krn workbook dibuka di Excel saat regenerasi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manuscript/A2-IRM_hasil_eksperimen.xlsx
+++ b/manuscript/A2-IRM_hasil_eksperimen.xlsx
@@ -9,18 +9,19 @@
   <sheets>
     <sheet name="0_Sampul" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="1_Ringkasan_Eksekutif" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2_Hasil_Utama_RMSE_MAE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3_Hybrid_vs_CF_Klasik" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="4_Signifikansi_Statistik" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5_Stabilitas_Variansi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="6_Data_Mentah_PerSeed" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="7_Dataset_dan_Hyperparameter" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2_Baseline_vs_Concat_Confidence" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3_Hasil_Utama_RMSE_MAE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4_Hybrid_vs_CF_Klasik" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5_Signifikansi_Statistik" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="6_Stabilitas_Variansi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="7_Data_Mentah_PerSeed" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="8_Dataset_dan_Hyperparameter" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2_Hasil_Utama_RMSE_MAE'!$A$3:$Q$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4_Signifikansi_Statistik'!$A$4:$J$94</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5_Stabilitas_Variansi'!$A$4:$L$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_Data_Mentah_PerSeed'!$A$3:$P$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3_Hasil_Utama_RMSE_MAE'!$A$3:$Q$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5_Signifikansi_Statistik'!$A$4:$J$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6_Stabilitas_Variansi'!$A$4:$L$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7_Data_Mentah_PerSeed'!$A$3:$P$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -364,6 +365,191 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>RMSE &amp; MAE: Baseline vs ABSA Concat+Confidence</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!B10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$A$11:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$B$11:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!C10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$A$11:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$C$11:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!D10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$A$11:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$D$11:$D$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!E10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$A$11:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2_Baseline_vs_Concat_Confidence'!$E$11:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Domain</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Error (RMSE / MAE)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>RMSE per Model per Domain</a:t>
             </a:r>
           </a:p>
@@ -379,7 +565,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!B27</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!B27</f>
             </strRef>
           </tx>
           <spPr>
@@ -389,12 +575,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!$A$28:$A$34</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!$A$28:$A$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!$B$28:$B$34</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!$B$28:$B$34</f>
             </numRef>
           </val>
         </ser>
@@ -403,7 +589,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!C27</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!C27</f>
             </strRef>
           </tx>
           <spPr>
@@ -413,12 +599,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!$A$28:$A$34</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!$A$28:$A$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!$C$28:$C$34</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!$C$28:$C$34</f>
             </numRef>
           </val>
         </ser>
@@ -427,7 +613,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!D27</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!D27</f>
             </strRef>
           </tx>
           <spPr>
@@ -437,12 +623,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!$A$28:$A$34</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!$A$28:$A$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2_Hasil_Utama_RMSE_MAE'!$D$28:$D$34</f>
+              <f>'3_Hasil_Utama_RMSE_MAE'!$D$28:$D$34</f>
             </numRef>
           </val>
         </ser>
@@ -512,7 +698,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
@@ -540,7 +726,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!B9</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!B9</f>
             </strRef>
           </tx>
           <spPr>
@@ -550,12 +736,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!$A$10:$A$12</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!$A$10:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!$B$10:$B$12</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!$B$10:$B$12</f>
             </numRef>
           </val>
         </ser>
@@ -564,7 +750,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!C9</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!C9</f>
             </strRef>
           </tx>
           <spPr>
@@ -574,12 +760,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!$A$10:$A$12</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!$A$10:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!$C$10:$C$12</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!$C$10:$C$12</f>
             </numRef>
           </val>
         </ser>
@@ -588,7 +774,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!D9</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!D9</f>
             </strRef>
           </tx>
           <spPr>
@@ -598,12 +784,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!$A$10:$A$12</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!$A$10:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'3_Hybrid_vs_CF_Klasik'!$D$10:$D$12</f>
+              <f>'4_Hybrid_vs_CF_Klasik'!$D$10:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -673,7 +859,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -699,7 +885,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'5_Stabilitas_Variansi'!B28</f>
+              <f>'6_Stabilitas_Variansi'!B28</f>
             </strRef>
           </tx>
           <spPr>
@@ -717,12 +903,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$A$29:$A$33</f>
+              <f>'6_Stabilitas_Variansi'!$A$29:$A$33</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$B$29:$B$33</f>
+              <f>'6_Stabilitas_Variansi'!$B$29:$B$33</f>
             </numRef>
           </val>
         </ser>
@@ -731,7 +917,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'5_Stabilitas_Variansi'!C28</f>
+              <f>'6_Stabilitas_Variansi'!C28</f>
             </strRef>
           </tx>
           <spPr>
@@ -749,162 +935,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$A$29:$A$33</f>
+              <f>'6_Stabilitas_Variansi'!$A$29:$A$33</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$C$29:$C$33</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Seed</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>RMSE</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>RMSE per Seed -- E-commerce (Amazon Electronics)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'5_Stabilitas_Variansi'!B36</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'5_Stabilitas_Variansi'!$A$37:$A$41</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'5_Stabilitas_Variansi'!$B$37:$B$41</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'5_Stabilitas_Variansi'!C36</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'5_Stabilitas_Variansi'!$A$37:$A$41</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'5_Stabilitas_Variansi'!$C$37:$C$41</f>
+              <f>'6_Stabilitas_Variansi'!$C$29:$C$33</f>
             </numRef>
           </val>
         </ser>
@@ -985,7 +1021,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>RMSE per Seed -- Hotel (TripAdvisor)</a:t>
+              <a:t>RMSE per Seed -- E-commerce (Amazon Electronics)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -999,7 +1035,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'5_Stabilitas_Variansi'!B44</f>
+              <f>'6_Stabilitas_Variansi'!B36</f>
             </strRef>
           </tx>
           <spPr>
@@ -1017,12 +1053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$A$45:$A$49</f>
+              <f>'6_Stabilitas_Variansi'!$A$37:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$B$45:$B$49</f>
+              <f>'6_Stabilitas_Variansi'!$B$37:$B$41</f>
             </numRef>
           </val>
         </ser>
@@ -1031,7 +1067,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'5_Stabilitas_Variansi'!C44</f>
+              <f>'6_Stabilitas_Variansi'!C36</f>
             </strRef>
           </tx>
           <spPr>
@@ -1049,12 +1085,162 @@
           </marker>
           <cat>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$A$45:$A$49</f>
+              <f>'6_Stabilitas_Variansi'!$A$37:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'5_Stabilitas_Variansi'!$C$45:$C$49</f>
+              <f>'6_Stabilitas_Variansi'!$C$37:$C$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Seed</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>RMSE</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>RMSE per Seed -- Hotel (TripAdvisor)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'6_Stabilitas_Variansi'!B44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'6_Stabilitas_Variansi'!$A$45:$A$49</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'6_Stabilitas_Variansi'!$B$45:$B$49</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'6_Stabilitas_Variansi'!C44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'6_Stabilitas_Variansi'!$A$45:$A$49</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'6_Stabilitas_Variansi'!$C$45:$C$49</f>
             </numRef>
           </val>
         </ser>
@@ -1156,6 +1342,33 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
@@ -1177,7 +1390,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1204,7 +1417,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1564,7 +1777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1580,7 +1793,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Digenerate: 2026-07-12</t>
+          <t>Digenerate: 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1814,7 @@
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Untuk kesimpulan, cukup baca Sheet 1-3 (tab warna HIJAU). Sheet 4 ke bawah (tab warna ABU-ABU) adalah lampiran teknis, tersedia kalau ingin menelusuri detail atau ada pertanyaan verifikasi.</t>
+          <t>Untuk kesimpulan, cukup baca Sheet 1-4 (tab warna HIJAU). Sheet 5 ke bawah (tab warna ABU-ABU) adalah lampiran teknis, tersedia kalau ingin menelusuri detail atau ada pertanyaan verifikasi.</t>
         </is>
       </c>
     </row>
@@ -1622,47 +1835,54 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>-&gt; 2_Hasil_Utama_RMSE_MAE: [WAJIB] Tabel RMSE/MAE lengkap 7 model x 3 domain</t>
+          <t>-&gt; 2_Baseline_vs_Concat_Confidence: [WAJIB] Fokus: baseline vs model terbaik (bukti klaim inti)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>-&gt; 3_Hybrid_vs_CF_Klasik: [WAJIB] Bukti model hybrid mengungguli CF klasik</t>
+          <t>-&gt; 3_Hasil_Utama_RMSE_MAE: [WAJIB] Tabel RMSE/MAE lengkap 7 model x 3 domain</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>-&gt; 4_Signifikansi_Statistik: [Lampiran] Detail uji Wilcoxon per seed</t>
+          <t>-&gt; 4_Hybrid_vs_CF_Klasik: [WAJIB] Bukti model hybrid mengungguli CF klasik</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>-&gt; 5_Stabilitas_Variansi: [Lampiran] Analisis stabilitas antar-seed</t>
+          <t>-&gt; 5_Signifikansi_Statistik: [Lampiran] Detail uji Wilcoxon per seed</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>-&gt; 6_Data_Mentah_PerSeed: [Lampiran] 105 baris data mentah per-seed</t>
+          <t>-&gt; 6_Stabilitas_Variansi: [Lampiran] Analisis stabilitas antar-seed</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>-&gt; 7_Dataset_dan_Hyperparameter: [Lampiran] Karakteristik dataset &amp; hyperparameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+          <t>-&gt; 7_Data_Mentah_PerSeed: [Lampiran] 105 baris data mentah per-seed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>-&gt; 8_Dataset_dan_Hyperparameter: [Lampiran] Karakteristik dataset &amp; hyperparameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Sumber data: checkpoints/results/ (lihat manuscript/A2-IRM_manuscript_draft.md utk metodologi lengkap dan draft manuskrip akademik).</t>
         </is>
@@ -1677,6 +1897,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1917,6 +2138,331 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F6F45"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fokus: Baseline vs Model Terbaik (ABSA Concat + Confidence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Perbandingan ini adalah klaim inti penelitian -- satu-satunya varian ABSA yang signifikan mengalahkan baseline di ketiga domain, sekaligus paling stabil antar-seed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>RMSE_Baseline</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>RMSE_ConcatConf</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Delta_RMSE_%</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>MAE_Baseline</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>MAE_ConcatConf</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Delta_MAE_%</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>SD_Baseline</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>SD_ConcatConf</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Faktor_Lebih_Stabil</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Seed_Signifikan</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>P_Value_Fisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Restoran (Yelp)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>0.6926</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.6791</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>0.5555</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>0.5505</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>5.472939685365184e-15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E-commerce (Amazon Electronics)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>0.6662</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>0.6516999999999999</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.4584</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>0.4386</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>1.573412688806018e-206</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hotel (TripAdvisor)</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>0.6501</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.6291</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>0.5252</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>0.5127</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>0.0217</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>1.235193072711498e-27</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>(Data pendukung grafik -- jangan diedit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RMSE Baseline</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RMSE Concat+Confidence</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MAE Baseline</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MAE Concat+Confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Restoran (Yelp)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.6926</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.6791</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5555</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.5505</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E-commerce (Amazon Electronics)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.6662</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.6516999999999999</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.4584</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.4386</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hotel (TripAdvisor)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.6501</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.6291</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5252</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.5127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F6F45"/>
@@ -3422,7 +3968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F6F45"/>
@@ -3651,7 +4197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="006E6E6E"/>
@@ -7351,7 +7897,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="006E6E6E"/>
@@ -8563,7 +9109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="006E6E6E"/>
@@ -14567,7 +15113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="006E6E6E"/>

</xml_diff>